<commit_message>
Versão do relatório v11 (11 out 2026): verificação das fontes, robustez complementar, resposta condicional do scaffold, stent sem vencedor universal, ecrã Como funciona e logótipo
</commit_message>
<xml_diff>
--- a/data/base_dados_biomateriais.xlsx
+++ b/data/base_dados_biomateriais.xlsx
@@ -443,7 +443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A155"/>
+  <dimension ref="A1:A182"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -510,7 +510,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>- Todos os valores são pontos de partida de manuais e revisões e estão marcados "A verificar".</t>
+          <t>- Os valores começaram como pontos de partida de manuais e revisões, marcados "A verificar"; cada valor confirmado na fonte passou a um dos estados "Verificado" (ver a Legenda). O número atual de valores verificados conta-se na coluna estado de materiais.csv (estados que começam por "Verificado").</t>
         </is>
       </c>
     </row>
@@ -627,7 +627,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>- Pt-Cr: cedência com fonte primária (O'Brien 2010, só resumo); módulo, tração e alongamento continuam "A verificar", com fontes secundárias na nota.</t>
+          <t>- Pt-Cr: cedência (480 MPa), módulo, tração e alongamento ficam "A verificar" (a cedência só foi lida no resumo de O'Brien 2010; estado mudado a 11 out 2026), com fontes secundárias na nota. Precisa de acesso: O'Brien BJ, Stinson JS, Larsen SR, Eppihimer MJ, Carroll WM. A platinum-chromium steel for cardiovascular stents. Biomaterials 2010;31:3755-3761 (doi:10.1016/j.biomaterials.2010.01.146), Tabelas 4 e 6; sem acesso aberto legítimo a 11 out 2026 (Unpaywall, Europe PMC, Semantic Scholar).</t>
         </is>
       </c>
     </row>
@@ -855,368 +855,360 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Legenda</t>
+          <t>Alterações v0.11 (10 out 2026): revisão por especialistas (frente DADOS)</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
+          <t>- Implante dentário: módulo do Ti-6Al-4V ELI (101-110, típico 105,5 GPa) e do Ti cp grau 4 (104,1 GPa) iguais aos valores verificados da haste (Li et al. 2014, Tabela 4); antes 110-114 e 103-110 GPa, "A verificar".</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
+          <t>- HA do scaffold: a porosidade passa a "A verificar" (o típico e o máximo não têm fonte) e o tempo de degradação ao novo estado "Valor de modelação". Os valores não mudam.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>- Estados da coluna estado:</t>
+          <t>- PLLA do stent: cedência e densidade com "[fonte a indicar]" (a referência anterior não tem estes números). Os valores não mudam.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
+          <t>- Notas: densidade do Ti-Zr (a confirmar), densidade do L605 (porque o típico é o da fita), níveis intermédios das rubricas, natureza dos valores de alongamento do stent.</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
-        </is>
-      </c>
+      <c r="A71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
+          <t>Alterações v0.12 (11 out 2026): decisões do André sobre a revisão</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+          <t>- Haste: o critério "Limite de fadiga (10^7 ciclos)" passa a "Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)" (materiais, critérios e perfis); os valores não mudam. Nota no Co-Cr-Mo: σmax acima de σ0,2 (tensão máxima a R = 0,1, não limite em amplitude). Ti-13Nb-13Zr e TNZT: modo de ensaio não registado (nota). Rótulo da norma do Co-Cr-Mo mantido, com a diferença anotada na cedência.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
+          <t>- Stent: cedência do 316L continua "A verificar" (nota com o mínimo de 190 MPa da Alleima, mínimo de especificação); L605 com a ressalva do Orsiro (60 e 80 µm) na espessura do strut, valor mantido (XIENCE); MP35N mantém o Resolute Integrity (nota).</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>- Teor de níquel (stent): % em massa; no WE43 é um limite máximo de impureza e tipico = máximo (pior caso).</t>
+          <t>- Perfis H-JOV e H-OST: notas sem efeito no ranking (fator 2 como valor de desenho; fixação no idoso com osteoporose).</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" t="inlineStr"/>
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>- Critérios do implante dentário: "Problema crítico do docente (2 out 2026)" passa a "Problema crítico indicado".</t>
+        </is>
+      </c>
     </row>
     <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
-        </is>
-      </c>
+      <c r="A77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+          <t>Alterações v0.13 (11 out 2026): verificação nas fontes primárias (stent e scaffold)</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" t="inlineStr"/>
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>- Stent: cedência do Pt-Cr (480 MPa) passa de "Verificado" a "A verificar" (só lida no resumo; precisa de acesso ao O'Brien 2010, Tabelas 4 e 6). Os valores não mudam.</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
+          <t>- Compósito PCL/β-TCP, resistência à compressão: 2,2 MPa (Kawai 2018, secção 3.4, cedência a 1 %, 59,5 %), "Verificado"; antes 2,2-6,38, típico 4,3 MPa. O 6,38 MPa (Wong 2025) sai: não é rastreável até uma fonte primária do compósito e não diz que grandeza é.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+          <t>- Compósito PCL/β-TCP, tempo de degradação: 26 meses (Zhong 2026, Discussão e Figura 7E-F, estimativa por correlação in vitro / in vivo), "Verificado"; antes 12-24, típico 18 meses (Rezwan 2006).</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
+          <t>- β-TCP poroso, tempo de degradação: 12,7 meses (5-26) (Hirata 2006, Resultados, 53 doentes), "Verificado"; antes 6-18, típico 12 meses.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>- Osteointegração (implante dentário; revista a 3 out 2026, pelo tipo e duração da evidência clínica do corpo do implante): 5 = coortes com 10 anos ou mais e milhares de implantes, mais meta-análises a 10 anos; 4 = ensaios aleatorizados ou meta-análises com centenas de implantes e pelo menos um estudo a 10 anos; 3 = meta-análises a 1-5 anos ou coortes de 10 anos pequenas e heterogéneas; 2 = uso clínico sem estudos clínicos dedicados (só equivalência em estudos animais); 1 = só evidência pré-clínica. Fontes por material na coluna referencia e em NOTAS_METODOLOGICAS.md.</t>
+          <t>- β-TCP poroso, módulo de compressão: 546 MPa (Montelongo 2021, 59,6 %), "Verificado"; antes 100-1000, típico 550 MPa.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>- Corrosão em meio oral (implante dentário, 3 out 2026): 5 = inerte em meio oral (sem corrosão eletroquímica nem degradação com efeito documentado); 4 = sem corrosão eletroquímica, mas com degradação lenta documentada em meio húmido ou oral (envelhecimento, absorção de água); 3 = metal passivo estável em saliva, atacado só em condições agressivas (fluoreto em meio ácido, tribocorrosão), com libertação de iões ou partículas documentada; 2 = metal atacado em condições orais comuns ou com acoplamento galvânico relevante; 1 = sem filme protetor estável.</t>
+          <t>- Efeito: no cenário A, o TOPSIS passa a pôr o β-TCP poroso em 1.º (o WASPAS e o VIKOR mantêm o compósito); no cenário B, os três métodos mantêm o compósito.</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" t="inlineStr">
-        <is>
-          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
-        </is>
-      </c>
+      <c r="A85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
+          <t>Alterações v0.14 (11 out 2026): análises de robustez complementares</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
+          <t>- Novo data/dimensoes_criterios.csv (caso, critério, dimensão, nota): mapa de cada critério dos casos quantitativos para uma dimensão (mecânica, biológica, clínica ou económica), usado só na análise de dupla contagem (scripts/robustez_extra.py). É uma escolha de desenho do trabalho, com a justificação na nota; os valores e os pesos da base não mudam.</t>
         </is>
       </c>
     </row>
     <row r="88">
-      <c r="A88" t="inlineStr">
-        <is>
-          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
-        </is>
-      </c>
+      <c r="A88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
+          <t>Legenda</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
+          <t>- min e max alimentam o Monte Carlo (distribuição entre mín. e máx.); nas propriedades dependentes da forma, só com valores da forma do dispositivo (regra da forma, v0.8).</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
+          <t>- tipico = valor usado nos métodos; por omissão o ponto médio; pode diferir quando a regra da forma ou outra regra o justifica, com nota.</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
+          <t>- Estados da coluna estado:</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
+          <t>- "A verificar": valor de partida (manual, revisão ou fonte secundária) ainda não confirmado na fonte original.</t>
         </is>
       </c>
     </row>
     <row r="94">
-      <c r="A94" t="inlineStr"/>
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>- "Verificado": valor confirmado na fonte indicada em doi_url (artigo ou norma).</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
+          <t>- "Verificado (fornecedor)": valor confirmado numa página de fornecedor que declara cumprir a norma, não no texto da norma.</t>
         </is>
       </c>
     </row>
     <row r="96">
-      <c r="A96" t="inlineStr"/>
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>- "Verificado (composição química)": valor que resulta da composição química do material (ex.: 0 % de níquel num polímero sem metais).</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Cuidados</t>
+          <t>- "Verificado (derivado)": valor calculado a partir de dados da fonte (ex.: razão σFS/σUTS × σUTS), com o cálculo na nota.</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
+          <t>- "Valor de modelação" (10 out 2026): número escolhido por uma regra do trabalho (ex.: tempo de degradação da HA, não reabsorvível, igual ao pior valor observado nos outros materiais, como a opção O2 do stent); a fonte confirma o comportamento (não reabsorve), não o número. Não conta como verificado nem entra na lista "A verificar".</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
+          <t>- Teor de níquel (stent): % em massa. No WE43 e no PLLA é 0 % pela composição nominal (decisão de 8 out 2026, ver "Funil de triagem"); o níquel da WE43 só aparece como impureza, até 0,005 %, e fica na nota.</t>
         </is>
       </c>
     </row>
     <row r="100">
-      <c r="A100" t="inlineStr">
-        <is>
-          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
-        </is>
-      </c>
+      <c r="A100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>4. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
+          <t>Tipos de critério (Petković et al., Appl Sci 2025;15:9198)</t>
         </is>
       </c>
     </row>
     <row r="102">
-      <c r="A102" t="inlineStr"/>
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Estrito = triagem passa/falha · Benefício = maior é melhor · Custo = menor é melhor · Alvo = mais próximo do valor-alvo é melhor</t>
+        </is>
+      </c>
     </row>
     <row r="103">
-      <c r="A103" t="inlineStr">
-        <is>
-          <t>Níveis de validação</t>
-        </is>
-      </c>
+      <c r="A103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
+          <t>Rubricas ordinais (1-5): justificar cada nota no relatório com uma referência</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" t="inlineStr"/>
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>- Corrosão: 5 = camada passiva estável sem libertação relevante; 3 = suscetível a picadas/fendas in vivo; 1 = corrosão clinicamente problemática</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>Perfis de doente (perfis_doente.csv)</t>
+          <t>- Segurança iónica/ALTR: 5 = sem contacto metal-metal; 4 = risco na junção cabeça-cone; 1 = libertação de iões Co/Cr com ALTR documentada</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Uma linha por regra (aprovada a 5 out 2026). Colunas: id, dispositivo, condicao (texto), condicao_codigo (condições</t>
+          <t>- Osteointegração (implante dentário; revista a 3 out 2026, pelo tipo e duração da evidência clínica do corpo do implante): 5 = coortes com 10 anos ou mais e milhares de implantes, mais meta-análises a 10 anos; 4 = ensaios aleatorizados ou meta-análises com centenas de implantes e pelo menos um estudo a 10 anos; 3 = meta-análises a 1-5 anos ou coortes de 10 anos pequenas e heterogéneas; 2 = uso clínico sem estudos clínicos dedicados (só equivalência em estudos animais); 1 = só evidência pré-clínica. Fontes por material na coluna referencia e em NOTAS_METODOLOGICAS.md.</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>separadas por "; ", todas têm de se verificar), efeito, alvo_do_efeito, valor, justificacao, fonte, doi_url, estado.</t>
+          <t>- Corrosão em meio oral (implante dentário, 3 out 2026): 5 = inerte em meio oral (sem corrosão eletroquímica nem degradação com efeito documentado); 4 = sem corrosão eletroquímica, mas com degradação lenta documentada em meio húmido ou oral (envelhecimento, absorção de água); 3 = metal passivo estável em saliva, atacado só em condições agressivas (fluoreto em meio ácido, tribocorrosão), com libertação de iões ou partículas documentada; 2 = metal atacado em condições orais comuns ou com acoplamento galvânico relevante; 1 = sem filme protetor estável.</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>- Efeitos: "peso multiplicado" (o peso do critério é multiplicado pelo valor e os pesos voltam a somar 1);</t>
+          <t>- Estética: 5 = cor de dente; 3 = neutro; 2 = sombra cinzenta possível</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>"critério acrescentado" (o critério entra com o peso do valor e os restantes ficam com 1 menos esse peso, na mesma</t>
+          <t>- Bioatividade (classificação de Hench): 5 = classe A, osteoprodutivo (ex.: vidro 45S5); 4 = classe B, osteocondutor com ligação química ao osso (HA, β-TCP); 3 = osteocondutor sem ligação química, ou compósito com fase bioativa minoritária; 2 = pouca interação; 1 = bioinerte ou sem osteocondução. Fonte: Hench LL. Bioactive ceramics: theory and clinical applications. Bioceramics 1994;7:3-14 (original não lido); classes A e B lidas em Bramhill J, Ross S, Ross G. Int J Environ Res Public Health 2017;14:66, doi:10.3390/ijerph14010066 (revisão, texto completo).</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>proporção); "leitura do problema" (P-foco com a leitura indicada e fator_foco_problema); "exclusão" (os materiais</t>
+          <t>- Imprimibilidade 3D: 5 = extrusão direta fácil; 3 = possível com limitações; 2 = requer técnicas especiais (robocasting, liofilização)</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>listados, separados por "; ", saem do ranking); "nota" (não altera o ranking; mostra o texto do alvo_do_efeito).</t>
+          <t>- Compatibilidade com RM: 5 = sem artefacto/aquecimento relevante; 4 = MR-condicional, artefacto pequeno (Ti); 3 = artefacto moderado (CoCr, Pt); 2 = artefacto marcado (aço inox)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>- Várias regras que sobem o mesmo critério: usa-se o maior fator, não o produto.</t>
+          <t>- Esterilização: 5 = aceita métodos padrão sem degradação; 4 = requer método específico sem perda de propriedades; 3 = método restrito com risco de degradação; 2 = degradação documentada</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>- Estado: "Verificado" = a fonte liga a condição (ou uma definição próxima, indicada na justificação) ao mecanismo do</t>
+          <t>- Custo relativo de material e fabrico (NÃO é preço clínico; critério de CUSTO): 1 = matéria-prima e processo maduros, menor complexidade; 2 = processo estabelecido com maior exigência de controlo; 3 = liga/material especializado ou cadeia de fabrico exigente; 4 = material caro, processo complexo, revestimento ou controlo rigoroso; 5 = material crítico, arquitetura complexa ou processo pouco escalável</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>critério; "Regra do trabalho" = a ligação ao critério é do trabalho, mesmo quando o fator de risco tem fonte. O</t>
+          <t>- Fabricabilidade: 5 = processos industriais maduros (incl. fabrico aditivo); 3 = possível com limitações; 2 = escala laboratorial</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>valor do fator é sempre de desenho. "A verificar" = a fonte não foi encontrada ou não liga a condição ao</t>
+          <t>- Galvânica cabeça-cone: 5 = sem par metálico; 3 = CoCr em cone de Ti (fretting documentado); 2 = múltiplas interfaces metal-metal</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>critério; a regra fica visível mas deve ser lida como provisória.</t>
+          <t>- Radiopacidade (stent): 5 = liga com fração elevada de elemento de Z alto (Pt-Cr); 4 = melhoria clara face ao 316L (L605, com W); 3 = referência dos metais de stent (316L, MP35N); 2 = pouco radiopaco (Nitinol); 1 = radiotransparente, precisa de marcadores (Mg WE43, PLLA). Critério: teor de elementos de Z alto (Pt, Z = 78; W, Z = 74). A densidade não é critério (desde a v0.3), serve só de evidência de apoio. Fontes: Allocco DJ et al. Trials 2010;11:1, doi:10.1186/1745-6215-11-1 (PMC2826324); PMC3692344 ("modest improvement" do CoCr face ao aço).</t>
         </is>
       </c>
     </row>
     <row r="118">
-      <c r="A118" t="inlineStr">
-        <is>
-          <t>- 8 out 2026: mais 25 regras (patologias: RM frequente, corticoterapia, insuficiência renal, artrite reumatoide,</t>
-        </is>
-      </c>
+      <c r="A118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>tabagismo, diabetes, radioterapia da cabeça e pescoço, osteoporose, idade avançada, hipertensão, alergia ao</t>
+          <t>- Níveis intermédios (2 e 4, quando não estão descritos na rubrica): usam-se quando o material fica entre duas descrições; a justificação de cada nota está na coluna notas ou referencia da linha do material em materiais.csv.</t>
         </is>
       </c>
     </row>
     <row r="120">
-      <c r="A120" t="inlineStr">
-        <is>
-          <t>cobalto e ao titânio); 42 regras no total. Mecanismo e o que cada fonte diz: docs/PATOLOGIAS_NOTAS.md.</t>
-        </is>
-      </c>
+      <c r="A120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>- Sem regra para o sexo: os dados demográficos só entram através de um mecanismo (docs/TP2_fisiopatologia_da_falha.md).</t>
+          <t>NOTA: índices ordinais só devem pesar ≤ 50 % do total de cada caso: o resto deve vir de propriedades medidas.</t>
         </is>
       </c>
     </row>
@@ -1226,225 +1218,402 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Funil de triagem (data/funil/, 8 out 2026)</t>
+          <t>Cuidados</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Três níveis, gerados por scripts/funil.py (results/funil.md e results/funil.csv):</t>
+          <t>1. Propriedades de scaffolds dependem da porosidade. Regra da porosidade: as propriedades mecânicas de um scaffold usam-se à porosidade típica desse material (±10 pontos percentuais); valores medidos a porosidades muito diferentes ficam de fora ou só alargam o intervalo, com nota. Dentro da janela, típico = mediana das fontes dentro da janela de porosidade (porosidade típica do material ±10 pontos percentuais); o intervalo vai do mínimo ao máximo dessas fontes. Regista sempre a porosidade e o método de fabrico do estudo.</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>1. Universo de partida: o resumo do Materials Project (dados abertos no AWS, versão 2026-09-28, licença CC BY 4.0;</t>
+          <t>2. Cerâmicos: resistência à flexão ≠ resistência à tração. Assinala sempre qual é.</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>atribuição: Jain A et al. APL Materials 2013;1:011002, doi:10.1063/1.4812323), os 118 elementos</t>
+          <t>3. Stents: o Nitinol é autoexpansível (outra classe): eliminado na triagem pela regra "Tipo de expansão"; só na discussão.</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>(elementos.csv, com a classificação de toxicidade de fontes oficiais) e as normas ASTM de materiais para implantes</t>
+          <t>4. Alongamento na rotura do stent: as fontes não dão todas o mesmo tipo de valor. No 316L, 40 % é típico (Alleima, coluna "typical"); no L605 e no MP35N, as fichas (Matthey, K-Tube) não dizem se 40 % é típico ou mínimo de especificação; no Pt-Cr, 45 % vem de uma fonte secundária. As diferenças entre ligas (40 contra 45 %) são da ordem da diferença entre mínimo e típico; o critério pesa 0,10 e o Monte Carlo aplica ±10 % aos valores únicos.</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>(normas.csv, com a norma como fonte).</t>
+          <t>5. Cenários (cenarios.csv): A = só materiais clínicos; B = inclui investigação e bioabsorvíveis. No stent, A = só permanentes em uso clínico (316L, L605, MP35N, Pt-Cr); B = A + Mg WE43 e PLLA.</t>
         </is>
       </c>
     </row>
     <row r="129">
-      <c r="A129" t="inlineStr">
-        <is>
-          <t>2. Filtros automáticos sobre o Materials Project (filtros.csv; os limites são valores de desenho): elementos</t>
-        </is>
-      </c>
+      <c r="A129" t="inlineStr"/>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>excluídos (radioativos, classe 1 da ICH Q3D, grupo 1 da IARC como elemento), estabilidade, densidade e módulo de</t>
+          <t>Níveis de validação</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Young (calculado a partir de K e G, E = 9KG/(3K + G)).</t>
+          <t>(1) verificação de código = reproduzir Petković et al. 2025; (2) robustez interna = cenários; (3) validação clínica = NÃO demonstrada (trabalho futuro).</t>
         </is>
       </c>
     </row>
     <row r="132">
-      <c r="A132" t="inlineStr">
-        <is>
-          <t>3. A base verificada (materiais.csv), onde se faz o MCDM.</t>
-        </is>
-      </c>
+      <c r="A132" t="inlineStr"/>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Cuidados: as propriedades do Materials Project são calculadas (DFT) e só servem para filtrar; nenhum valor do Materials</t>
+          <t>Perfis de doente (perfis_doente.csv)</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Project entra no MCDM. O Materials Project só tem fases cristalinas ordenadas (as ligas como o Ti-6Al-4V e os polímeros</t>
+          <t>Uma linha por regra (aprovada a 5 out 2026). Colunas: id, dispositivo, condicao (texto), condicao_codigo (condições</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>não estão lá); por isso o nível 3 não sai automaticamente do nível 2: junta os materiais com norma ou uso clínico e</t>
+          <t>separadas por "; ", todas têm de se verificar), efeito, alvo_do_efeito, valor, justificacao, fonte, doi_url, estado.</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>propriedades confirmadas em fontes. Não se copiam dados do MatWeb nem do ASM (termos de uso); podem ser citados como</t>
+          <t>- Efeitos: "peso multiplicado" (o peso do critério é multiplicado pelo valor e os pesos voltam a somar 1);</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>fontes de consulta.</t>
+          <t>"critério acrescentado" (o critério entra com o peso do valor e os restantes ficam com 1 menos esse peso, na mesma</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>- Níquel (decisão de 8 out 2026): 0 % no PLLA e na liga de Mg WE43, pela composição nominal (o níquel da WE43 só</t>
+          <t>proporção); "leitura do problema" (P-foco com a leitura indicada e fator_foco_problema); "exclusão" (os materiais</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>aparece como impureza, até 0,005 %). Num critério de custo com mínimo 0, o WASPAS usa a eq. 11 de Petković et al.</t>
+          <t>listados, separados por "; ", saem do ranking); "nota" (não altera o ranking; mostra o texto do alvo_do_efeito).</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>com o alvo T = 0 (r = 1 - x / máx), porque a eq. 10 (mín / x) fica indefinida; o perfil de alergia ao níquel passa</t>
+          <t>- Várias regras que sobem o mesmo critério: usa-se o maior fator, não o produto.</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>a funcionar no cenário B. Nenhum critério dos casos de base tem mínimo 0, por isso os rankings do relatório não</t>
+          <t>- Estado: "Verificado" = a fonte liga a condição (ou uma definição próxima, indicada na justificação) ao mecanismo do</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>mudam (confirmado: results/pontuacoes.csv igual).</t>
+          <t>critério; "Regra do trabalho" = a ligação ao critério é do trabalho, mesmo quando o fator de risco tem fonte. O</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>- H1 (jovem ativo) e H3 (IMC 38) dão o mesmo ranking: as duas regras sobem só o limite de fadiga com fator 2, porque</t>
+          <t>valor do fator é sempre de desenho. "A verificar" = a fonte não foi encontrada ou não liga a condição ao</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>ambas significam mais carga cíclica (decisão de 8 out 2026: fica assim; a aplicação explica-o).</t>
+          <t>critério; a regra fica visível mas deve ser lida como provisória.</t>
         </is>
       </c>
     </row>
     <row r="145">
-      <c r="A145" t="inlineStr"/>
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>- 8 out 2026: mais 25 regras (patologias: RM frequente, corticoterapia, insuficiência renal, artrite reumatoide,</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Filtros de requisito (filtros_material.csv, 8 out 2026)</t>
+          <t>tabagismo, diabetes, radioterapia da cabeça e pescoço, osteoporose, idade avançada, hipertensão, alergia ao</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Uma linha por material: ferromagnetico (sim, não ou A verificar; fonte_rm), vapor, oxido_etileno e radiacao_gama</t>
+          <t>cobalto e ao titânio); 42 regras no total. Mecanismo e o que cada fonte diz: docs/PATOLOGIAS_NOTAS.md.</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>(compatível, com restrições, incompatível ou A verificar; fonte_esterilizacao), notas e estado (Verificado quando os</t>
+          <t>- Sem regra para o sexo: os dados demográficos só entram através de um mecanismo (docs/TP2_fisiopatologia_da_falha.md).</t>
         </is>
       </c>
     </row>
     <row r="149">
-      <c r="A149" t="inlineStr">
-        <is>
-          <t>quatro campos têm fonte, Parcial quando só alguns têm, A verificar quando nenhum tem). Decisão de 8 out 2026: a</t>
-        </is>
-      </c>
+      <c r="A149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>ISO 10993-1, a RM (ASTM F2503) e a esterilização entram como filtros e no texto, não como critérios com peso, para não</t>
+          <t>Funil de triagem (data/funil/, 8 out 2026)</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>mudar os rankings do relatório; a esterilização tem também um cenário de sensibilidade (método imposto; saem os</t>
+          <t>Três níveis, gerados por scripts/funil.py (results/funil.md e results/funil.csv):</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>incompatíveis). Resultado em results/filtros.md (src/biomat_mcdm/filtros.py, chamado pelo run_all.py). Cuidados: a</t>
+          <t>1. Universo de partida: o resumo do Materials Project (dados abertos no AWS, versão 2026-09-28, licença CC BY 4.0;</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>compatibilidade dos metais com vapor e gama assenta numa frase genérica (Yu et al. 2026) e nenhuma liga foi testada em</t>
+          <t>atribuição: Jain A et al. APL Materials 2013;1:011002, doi:10.1063/1.4812323), os 118 elementos</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>particular; o óxido de etileno ficou A verificar nos metais; o "incompatível" da WE43 com vapor vem de um só provete</t>
+          <t>(elementos.csv, com a classificação de toxicidade de fontes oficiais) e as normas ASTM de materiais para implantes</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
+        <is>
+          <t>(normas.csv, com a norma como fonte).</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>2. Filtros automáticos sobre o Materials Project (filtros.csv; os limites são valores de desenho): elementos</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>excluídos (radioativos, classe 1 da ICH Q3D, grupo 1 da IARC como elemento), estabilidade, densidade e módulo de</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Young (calculado a partir de K e G, E = 9KG/(3K + G)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>3. A base verificada (materiais.csv), onde se faz o MCDM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Cuidados: as propriedades do Materials Project são calculadas (DFT) e só servem para filtrar; nenhum valor do Materials</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Project entra no MCDM. O Materials Project só tem fases cristalinas ordenadas (as ligas como o Ti-6Al-4V e os polímeros</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>não estão lá); por isso o nível 3 não sai automaticamente do nível 2: junta os materiais com norma ou uso clínico e</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>propriedades confirmadas em fontes. Não se copiam dados do MatWeb nem do ASM (termos de uso); podem ser citados como</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>fontes de consulta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>- Níquel (decisão de 8 out 2026): 0 % no PLLA e na liga de Mg WE43, pela composição nominal (o níquel da WE43 só</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>aparece como impureza, até 0,005 %). Num critério de custo com mínimo 0, o WASPAS usa a eq. 11 de Petković et al.</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>com o alvo T = 0 (r = 1 - x / máx), porque a eq. 10 (mín / x) fica indefinida; o perfil de alergia ao níquel passa</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>a funcionar no cenário B. Nenhum critério dos casos de base tem mínimo 0, por isso os rankings do relatório não</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>mudam (confirmado: results/pontuacoes.csv igual).</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>- H1 (jovem ativo) e H3 (IMC 38) dão o mesmo ranking: as duas regras sobem só a resistência à fadiga com fator 2, porque</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>ambas significam mais carga cíclica (decisão de 8 out 2026: fica assim; a aplicação explica-o).</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Filtros de requisito (filtros_material.csv, 8 out 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Uma linha por material: ferromagnetico (sim, não ou A verificar; fonte_rm), vapor, oxido_etileno e radiacao_gama</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>(compatível, com restrições, incompatível ou A verificar; fonte_esterilizacao), notas e estado (Verificado quando os</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>quatro campos têm fonte, Parcial quando só alguns têm, A verificar quando nenhum tem). Decisão de 8 out 2026: a</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>ISO 10993-1, a RM (ASTM F2503) e a esterilização entram como filtros e no texto, não como critérios com peso, para não</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>mudar os rankings do relatório; a esterilização tem também um cenário de sensibilidade (método imposto; saem os</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>incompatíveis). Resultado em results/filtros.md (src/biomat_mcdm/filtros.py, chamado pelo run_all.py). Cuidados: a</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>compatibilidade dos metais com vapor e gama assenta numa frase genérica (Yu et al. 2026) e nenhuma liga foi testada em</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>particular; o óxido de etileno ficou A verificar nos metais; o "incompatível" da WE43 com vapor vem de um só provete</t>
+        </is>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
         <is>
           <t>(Becerra 2021); o 316L encruado pode ter magnetização fraca [confirmar].</t>
         </is>
@@ -2426,7 +2595,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2731,7 +2900,7 @@
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Forjado a quente; Okazaki 2012, Tabela 2: σ0,2 = 669 ± 40 MPa (mín.-máx. = média ± DP)</t>
+          <t>Forjado a quente; Okazaki 2012, Tabela 2: σ0,2 = 669 ± 40 MPa (mín.-máx. = média ± DP); rótulo da norma mantido (ASTM F799/F1537; decisão de 11 out 2026): o valor de Okazaki 2012 é de Co-Cr-Mo forjado a quente e pode ficar abaixo do mínimo de cedência de especificação da ASTM F799 (mínimo não lido na norma); a diferença fica anotada e não muda o valor</t>
         </is>
       </c>
       <c r="N9" t="n">
@@ -2842,7 +3011,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -2868,7 +3037,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Forjado a quente; Okazaki 2012, Tabela 2: σFS/σUTS = 0,74 e σUTS = 1075 ± 20 MPa; cálculo: 0,74 × 1075 = 796 MPa; ensaio tração-tração, R = 0,1, 10 Hz, meio de Eagle a 37 °C</t>
+          <t>Forjado a quente; Okazaki 2012, Tabela 2: σFS/σUTS = 0,74 e σUTS = 1075 ± 20 MPa; cálculo: 0,74 × 1075 = 796 MPa; ensaio tração-tração, R = 0,1, 10 Hz, meio de Eagle a 37 °C; σmax &gt; σ0,2 no Co-Cr-Mo: é a tensão máxima de um ensaio tração-tração (R = 0,1), não um limite em amplitude (amplitude 0,45 × σmax)</t>
         </is>
       </c>
       <c r="N11" t="n">
@@ -3253,7 +3422,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -3659,7 +3828,7 @@
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -4070,7 +4239,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -4091,7 +4260,7 @@
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Liga β sem Al/V, módulo mais baixo</t>
+          <t>Liga β sem Al/V, módulo mais baixo; modo de ensaio (R, meio, frequência) não indicado nesta linha: pode não ser comparável com os valores de Okazaki 2012 (R = 0,1); ver a secção 9.9 do relatório</t>
         </is>
       </c>
       <c r="N29" t="n">
@@ -4476,7 +4645,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -4502,7 +4671,7 @@
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Excluído no cenário 'só materiais clínicos'; variante com 0,06 % de O; Li et al. 2014, secção 4.1 (texto): 275 MPa, solubilizado; o valor de 450 MPa corresponde à variante com mais oxigénio (0,46 % O)</t>
+          <t>Excluído no cenário 'só materiais clínicos'; variante com 0,06 % de O; Li et al. 2014, secção 4.1 (texto): 275 MPa, solubilizado; o valor de 450 MPa corresponde à variante com mais oxigénio (0,46 % O); modo de ensaio (R) não registado nesta linha: pode não ser comparável com os valores de Okazaki 2012 (R = 0,1); ver a secção 9.9 do relatório</t>
         </is>
       </c>
       <c r="N35" t="n">
@@ -5728,22 +5897,32 @@
         </is>
       </c>
       <c r="I53" t="n">
-        <v>103</v>
+        <v>104.1</v>
       </c>
       <c r="J53" t="n">
-        <v>110</v>
+        <v>104.1</v>
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>Li et al. 2014, Tabela 4 (cita Niinomi 1998): 104,1 GPa, recozido; o mesmo valor verificado da haste (mesma liga e norma); a ASTM F67 não especifica módulo: mín. = máx. = típico; valor anterior: 103-110 GPa, típico 106,5 (Niinomi 1998, A verificar)</t>
         </is>
       </c>
       <c r="N53" t="n">
-        <v>106.5</v>
+        <v>104.1</v>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -6109,22 +6288,32 @@
         </is>
       </c>
       <c r="I59" t="n">
+        <v>101</v>
+      </c>
+      <c r="J59" t="n">
         <v>110</v>
       </c>
-      <c r="J59" t="n">
-        <v>114</v>
-      </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>Niinomi M. Mater Sci Eng A 1998;243:231-236</t>
+          <t>Li Y et al. Materials 2014;7:1709 (New Developments of Ti-Based Alloys for Biomedical Applications)</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.3390/ma7031709</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>Li et al. 2014, Tabela 4 (cita Niinomi 1998): 101-110 GPa, recozido; típico = ponto médio; o mesmo valor verificado da haste (mesma liga e norma); valor anterior: 110-114 GPa, típico 112 (era do Ti-6Al-4V normal, ASTM F1472, Li 2014, Tabela 4)</t>
         </is>
       </c>
       <c r="N59" t="n">
-        <v>112</v>
+        <v>105.5</v>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -6678,6 +6867,11 @@
           <t>Ficha técnica do fabricante (ex.: Straumann Roxolid): confirmar</t>
         </is>
       </c>
+      <c r="M68" t="inlineStr">
+        <is>
+          <t>valor a confirmar: parece copiado do Ti-13Nb-13Zr; pela regra das misturas em massa (Ti 4,51 e Zr 6,52 g/cm³, 15 % de Zr) daria cerca de 4,73 g/cm³ (cálculo aproximado, não é fonte); não é critério do dentário desde a v0.10</t>
+        </is>
+      </c>
       <c r="N68" t="n">
         <v>5</v>
       </c>
@@ -7704,6 +7898,11 @@
           <t>Hanawa T. J Artif Organs 2009;12:73-79 (metais para stents)</t>
         </is>
       </c>
+      <c r="M84" t="inlineStr">
+        <is>
+          <t>fica A verificar (decisão de 11 out 2026): a ficha Alleima 316LVM (tubo de parede fina recozido, lida a 10 out 2026) dá Rp0,2 = 190 MPa como mínimo de especificação, não como valor típico, por isso não substitui o intervalo; para registo: tubo de parede grossa recozido 220 MPa (mín.)</t>
+        </is>
+      </c>
       <c r="N84" t="n">
         <v>272.5</v>
       </c>
@@ -8045,12 +8244,12 @@
       </c>
       <c r="M89" t="inlineStr">
         <is>
-          <t>Permanente: só entra no cenário B como 'não reabsorve'</t>
+          <t>Permanente: só entra no cenário B como 'não reabsorve'; valor de modelação: sem valor na base, nos métodos recebe o pior valor observado (48 meses, máximo do PLLA; regra da secção 2.4 do relatório)</t>
         </is>
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -8454,7 +8653,7 @@
       </c>
       <c r="M95" t="inlineStr">
         <is>
-          <t>mín.: 9,07 g/cm³ (Haynes, HAYNES 25, https://haynesintl.com/en/alloys/alloy-portfolio/high-temperature-alloys/haynes-25/); típico e máx.: 9,27 g/cm³ (Matthey, fita); valor anterior: 9,1 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>mín.: 9,07 g/cm³ (Haynes, HAYNES 25, https://haynesintl.com/en/alloys/alloy-portfolio/high-temperature-alloys/haynes-25/); típico e máx.: 9,27 g/cm³ (Matthey, fita); o típico é o máximo do intervalo porque a fita é a forma do dispositivo (como na regra da forma); o mínimo vem de outra ficha (Haynes); não entra no ranking do stent; valor anterior: 9,1 g/cm³ (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N95" t="n">
@@ -8525,7 +8724,7 @@
       </c>
       <c r="M96" t="inlineStr">
         <is>
-          <t>XIENCE V / MULTI-LINK VISION: 81 µm; revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; material L-605 confirmado no FDA SSED P070015 (https://www.accessdata.fda.gov/cdrh_docs/pdf7/P070015b.pdf); Brami 2023: https://doi.org/10.3390/jcm12216711; valor anterior: 60-90 µm (Hanawa 2009)</t>
+          <t>XIENCE V / MULTI-LINK VISION: 81 µm; revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; material L-605 confirmado no FDA SSED P070015 (https://www.accessdata.fda.gov/cdrh_docs/pdf7/P070015b.pdf); Brami 2023: https://doi.org/10.3390/jcm12216711; valor anterior: 60-90 µm (Hanawa 2009); ressalva (decisão de 11 out 2026, valor mantido): há DES de L605 com struts mais finos, Orsiro Mission 60 µm (2,25-3,0 mm) e 80 µm (3,5-4,0 mm), ficha Teleflex/Biotronik nov 2025 (https://go.teleflex.com/rs/114-ZNV-758/images/Orsiro_Mission_Spec_Sheet_EN_Nov.2025_TFX.pdf, lida a 11 out 2026); a vantagem do Pt-Cr neste critério é do dispositivo escolhido, não da liga</t>
         </is>
       </c>
       <c r="N96" t="n">
@@ -8585,12 +8784,12 @@
       </c>
       <c r="M97" t="inlineStr">
         <is>
-          <t>Permanente: só entra no cenário B como 'não reabsorve'</t>
+          <t>Permanente: só entra no cenário B como 'não reabsorve'; valor de modelação: sem valor na base, nos métodos recebe o pior valor observado (48 meses, máximo do PLLA; regra da secção 2.4 do relatório)</t>
         </is>
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -9065,7 +9264,7 @@
       </c>
       <c r="M104" t="inlineStr">
         <is>
-          <t>Resolute Integrity 90 µm (Brami 2023); Driver 91 µm (Macaya-Ten 2024); revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; MP35N no Resolute Integrity confirmado no FDA SSED P110013 (https://www.accessdata.fda.gov/cdrh_docs/pdf11/P110013b.pdf); valor anterior: 60-90 µm (Hanawa 2009)</t>
+          <t>Resolute Integrity 90 µm (Brami 2023); Driver 91 µm (Macaya-Ten 2024); revisões (Brami 2023; Macaya-Ten 2024) que citam o fabricante; espessura de strut = propriedade do dispositivo, não do material; MP35N no Resolute Integrity confirmado no FDA SSED P110013 (https://www.accessdata.fda.gov/cdrh_docs/pdf11/P110013b.pdf); valor anterior: 60-90 µm (Hanawa 2009); dispositivo mantido: Resolute Integrity (decisão de 11 out 2026); as plataformas atuais da mesma família (Onyx, com núcleo de platina-irídio segundo a página da Medtronic lida a 10 out 2026) não foram avaliadas; espessura do Onyx por confirmar</t>
         </is>
       </c>
       <c r="N104" t="n">
@@ -9125,12 +9324,12 @@
       </c>
       <c r="M105" t="inlineStr">
         <is>
-          <t>Permanente: só entra no cenário B como 'não reabsorve'</t>
+          <t>Permanente: só entra no cenário B como 'não reabsorve'; valor de modelação: sem valor na base, nos métodos recebe o pior valor observado (48 meses, máximo do PLLA; regra da secção 2.4 do relatório)</t>
         </is>
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -9250,7 +9449,7 @@
       </c>
       <c r="M107" t="inlineStr">
         <is>
-          <t>Alta radiopacidade; fontes secundárias (lidas em texto completo a 8 out 2026): Huibregtse 2011, Tabela 1: 203 GPa; Samant 2021, Tabela suplementar 1: 203 GPa; ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6, sem acesso; o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
+          <t>Alta radiopacidade; fontes secundárias (lidas em texto completo a 8 out 2026): Huibregtse 2011, Tabela 1: 203 GPa; Samant 2021, Tabela suplementar 1: 203 GPa; ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6; precisa de acesso: procura de 11 out 2026 sem acesso aberto legítimo (Unpaywall: closed; Europe PMC: só por assinatura; Semantic Scholar: closed; sem versão de autor encontrada; Allocco 2010, PMC2826324, só dá a composição); o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
         </is>
       </c>
       <c r="N107" t="n">
@@ -9321,7 +9520,7 @@
       </c>
       <c r="M108" t="inlineStr">
         <is>
-          <t>só resumo; valor anterior: 480 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
+          <t>só resumo (o valor do resumo coincide, mas não foi lido no texto completo nem na tabela); precisa de acesso: O'Brien 2010, Tabelas 4 e 6, sem acesso aberto legítimo (procura de 11 out 2026); estado mudado de Verificado para A verificar a 11 out 2026; valor anterior: 480 MPa (Hanawa T. J Artif Organs 2009;12:73-79)</t>
         </is>
       </c>
       <c r="N108" t="n">
@@ -9329,7 +9528,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -9392,7 +9591,7 @@
       </c>
       <c r="M109" t="inlineStr">
         <is>
-          <t>fontes secundárias (lidas em texto completo a 8 out 2026): Huibregtse 2011, Tabela 1: 834 MPa; Samant 2021, Tabela suplementar 1: 834 MPa; ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6, sem acesso; o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
+          <t>fontes secundárias (lidas em texto completo a 8 out 2026): Huibregtse 2011, Tabela 1: 834 MPa; Samant 2021, Tabela suplementar 1: 834 MPa; ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6; precisa de acesso: procura de 11 out 2026 sem acesso aberto legítimo (Unpaywall: closed; Europe PMC: só por assinatura; Semantic Scholar: closed; sem versão de autor encontrada; Allocco 2010, PMC2826324, só dá a composição); o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
         </is>
       </c>
       <c r="N109" t="n">
@@ -9463,7 +9662,7 @@
       </c>
       <c r="M110" t="inlineStr">
         <is>
-          <t>fontes secundárias (lidas em texto completo a 8 out 2026): Samant 2021, Tabela suplementar 1: 45 % (a única fonte encontrada com o alongamento); ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6, sem acesso; o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
+          <t>fontes secundárias (lidas em texto completo a 8 out 2026): Samant 2021, Tabela suplementar 1: 45 % (a única fonte encontrada com o alongamento); ambas remetem para O'Brien BJ et al. Biomaterials 2010;31:3755-3761 (Tabelas 4 e 6; precisa de acesso: procura de 11 out 2026 sem acesso aberto legítimo (Unpaywall: closed; Europe PMC: só por assinatura; Semantic Scholar: closed; sem versão de autor encontrada; Allocco 2010, PMC2826324, só dá a composição); o resumo só dá a cedência); as fichas da FDA (SSED P110010, P100023, P150003) dizem só que a tração, a cedência e o alongamento cumprem a especificação, sem números; o Hanawa 2009 (citado antes) é anterior ao Pt-Cr e o resumo não o refere; Huibregtse e Samant têm financiamento ou coautores da Boston Scientific</t>
         </is>
       </c>
       <c r="N110" t="n">
@@ -9665,12 +9864,12 @@
       </c>
       <c r="M113" t="inlineStr">
         <is>
-          <t>Permanente: só entra no cenário B como 'não reabsorve'</t>
+          <t>Permanente: só entra no cenário B como 'não reabsorve'; valor de modelação: sem valor na base, nos métodos recebe o pior valor observado (48 meses, máximo do PLLA; regra da secção 2.4 do relatório)</t>
         </is>
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -10150,12 +10349,12 @@
       </c>
       <c r="M121" t="inlineStr">
         <is>
-          <t>Permanente: só entra no cenário B como 'não reabsorve'</t>
+          <t>Permanente: só entra no cenário B como 'não reabsorve'; valor de modelação: sem valor na base, nos métodos recebe o pior valor observado (48 meses, máximo do PLLA; regra da secção 2.4 do relatório)</t>
         </is>
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -10880,7 +11079,12 @@
       </c>
       <c r="K132" t="inlineStr">
         <is>
-          <t>Ensaios ABSORB / comunicação FDA 2017 (Absorb BVS)</t>
+          <t>[fonte a indicar] (antes: ensaios ABSORB / comunicação FDA 2017)</t>
+        </is>
+      </c>
+      <c r="M132" t="inlineStr">
+        <is>
+          <t>fonte a indicar: a referência anterior (ensaios ABSORB / comunicação FDA 2017) não tem estes números (ver a nota do módulo); Ang HY et al. J Thorac Dis 2017, Tabela 1 (PMC5583085, lida a 10 out 2026) não dá a cedência do PLLA, só módulo, resistência e alongamento; procura de 11 out 2026 na Europe PMC (acesso aberto) sem fonte primária com a cedência do PLLA de stents</t>
         </is>
       </c>
       <c r="N132" t="n">
@@ -11083,7 +11287,12 @@
       </c>
       <c r="K135" t="inlineStr">
         <is>
-          <t>Ensaios ABSORB / comunicação FDA 2017 (Absorb BVS)</t>
+          <t>[fonte a indicar] (antes: ensaios ABSORB / comunicação FDA 2017)</t>
+        </is>
+      </c>
+      <c r="M135" t="inlineStr">
+        <is>
+          <t>fonte a indicar: a referência anterior (ensaios ABSORB / comunicação FDA 2017) não tem estes números (ver a nota do módulo); Ang HY et al. J Thorac Dis 2017, Tabela 1 (PMC5583085, lida a 10 out 2026) não dá a densidade; não entra no ranking do stent</t>
         </is>
       </c>
       <c r="N135" t="n">
@@ -12713,7 +12922,7 @@
       </c>
       <c r="M159" t="inlineStr">
         <is>
-          <t>Pro Osteon 200 (HA coralina): porosidade 57 %, resistência à compressão 5,8 MPa (4-10 MPa), conferido no PDF do 510(k); blocos sinterizados com 56 % de macroporosidade (Hoogendoorn 1984, só resumo); o típico de 65 % e o máximo de 80 % não têm fonte própria; valor anterior: 50-80 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>Pro Osteon 200 (HA coralina): porosidade 57 %, resistência à compressão 5,8 MPa (4-10 MPa), conferido no PDF do 510(k); blocos sinterizados com 56 % de macroporosidade (Hoogendoorn 1984, só resumo); o típico de 65 % e o máximo de 80 % não têm fonte própria; valor anterior: 50-80 % (Karageorgiou V, Kaplan D. Biomaterials 2005;26); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA; estado passou de "Verificado (fornecedor)" a "A verificar" a 10 out 2026, porque o típico e o máximo não têm fonte (conferido só o 57 % do Pro Osteon no 510(k))</t>
         </is>
       </c>
       <c r="N159" t="n">
@@ -12721,7 +12930,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>Verificado (fornecedor)</t>
+          <t>A verificar</t>
         </is>
       </c>
     </row>
@@ -12784,7 +12993,7 @@
       </c>
       <c r="M160" t="inlineStr">
         <is>
-          <t>não reabsorvível; valor de modelação, como a opção O2 do stent: mínimo 42 meses (sem reabsorção mensurável em 3,5 anos, cão, blocos com 56 % de macroporosidade, Hoogendoorn 1984; "not resorbed at all", coelho, Oonishi 2000; só resumo nos dois); máximo e típico = pior valor observado nos outros materiais do scaffold (60 meses, PLLA); valor anterior: 24-60 meses (Rezwan K et al. Biomaterials 2006;27); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>não reabsorvível; valor de modelação, como a opção O2 do stent: mínimo 42 meses (sem reabsorção mensurável em 3,5 anos, cão, blocos com 56 % de macroporosidade, Hoogendoorn 1984; "not resorbed at all", coelho, Oonishi 2000; só resumo nos dois); máximo e típico = pior valor observado nos outros materiais do scaffold (60 meses, PLLA); valor anterior: 24-60 meses (Rezwan K et al. Biomaterials 2006;27); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA; estado passou de "Verificado" a "Valor de modelação" a 10 out 2026 (as fontes confirmam a não reabsorção, não os números)</t>
         </is>
       </c>
       <c r="N160" t="n">
@@ -12792,7 +13001,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>Verificado</t>
+          <t>Valor de modelação</t>
         </is>
       </c>
     </row>
@@ -13046,27 +13255,32 @@
         </is>
       </c>
       <c r="I164" t="n">
-        <v>100</v>
+        <v>546</v>
       </c>
       <c r="J164" t="n">
-        <v>1000</v>
+        <v>546</v>
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Montelongo SA et al. J Mater Sci Mater Med 2021;32:94 (Resultados, grupo da ponta de 200 µm)</t>
+        </is>
+      </c>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s10856-021-06569-9</t>
         </is>
       </c>
       <c r="M164" t="inlineStr">
         <is>
-          <t>uma só fonte na janela de porosidade: 546 MPa a 59,6 % (Montelongo 2021, texto completo, https://doi.org/10.1007/s10856-021-06569-9); o intervalo 100-1000 MPa continua a vir da revisão; Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>uma só fonte na janela de porosidade (texto completo, PMC8364524): "elastic modulus (545.82 ± 72.93 MPa)" a 59,6 % de porosidade (ponta de 200 µm); os outros grupos (924 e cerca de 696 MPa) têm 45-55 %, fora da janela; confirma o típico da base; diferença registada a 11 out 2026: intervalo anterior 100-1000, típico 550 MPa (Rezwan K et al. Biomaterials 2006;27:3413-3431, revisão, sem fonte primária para o intervalo); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N164" t="n">
-        <v>550</v>
+        <v>546</v>
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -13183,27 +13397,32 @@
         </is>
       </c>
       <c r="I166" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="J166" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Hirata M et al. Int Orthop 2006;30:510-513 (Resultados)</t>
+        </is>
+      </c>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1007/s00264-006-0156-1</t>
         </is>
       </c>
       <c r="M166" t="inlineStr">
         <is>
-          <t>Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
+          <t>β-TCP purificado (Osferion), 75 % de porosidade, 53 doentes, radiografia (texto completo, PMC3172745): "The mean period to complete resorption of the material was 12.7 (5–26) months"; ressalvas: média só dos 23 casos (43 %) com reabsorção completa, os restantes 57 % ainda tinham material no fim do seguimento; depende do volume e da forma (grânulos ou bloco); confirma a ordem de grandeza da base; diferença registada a 11 out 2026: intervalo anterior 6-18, típico 12 meses (Rezwan K et al. Biomaterials 2006;27:3413-3431, revisão); Estatuto [confirmar]: Rezwan et al. 2006; Bose et al. 2012; base 510(k) da FDA</t>
         </is>
       </c>
       <c r="N166" t="n">
-        <v>12</v>
+        <v>12.7</v>
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -13795,11 +14014,11 @@
         <v>2.2</v>
       </c>
       <c r="J175" t="n">
-        <v>6.38</v>
+        <v>2.2</v>
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>Kawai T et al. J Orthop Res 2018;36:1002-1011; Wong WS et al. Cureus 2025;17:e86272</t>
+          <t>Kawai T et al. J Orthop Res 2018;36:1002-1011 (secção 3.4 e Figura 2C)</t>
         </is>
       </c>
       <c r="L175" t="inlineStr">
@@ -13809,15 +14028,15 @@
       </c>
       <c r="M175" t="inlineStr">
         <is>
-          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão: a verificar, duas fontes fracas: 2,2 MPa a 59,5 %, no limite inferior da janela (Kawai 2018, texto completo); 6,38 MPa a 70 % (Wong 2025, fonte secundária, https://doi.org/10.7759/cureus.86272); típico = ponto médio; de fora: 27,9 MPa em Wang 2024, que não é tensão de cedência (o Wang 2024 foi retirado de toda a base a 3 out 2026: Editor Note da revista, ver o módulo); valor anterior: 3-12 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>regra da porosidade (típico do PCL/β-TCP: 70 %, janela 60-80 %), PCL/TCP 80:20 por FDM ou extrusão: 2,2 MPa, cedência a 1 % de desvio, a 59,5 % de porosidade (Kawai 2018, texto completo, PMC5924591, secção 3.4: "the average strength of the 60% porous scaffold was 2.2 MPa"; ensaio na secção 2.4.1); apoio: Bruyas A et al. J Mater Res 2018;33:1948-1959 (PMC6197810, Figura 7c, leitura de figura): cerca de 2,2 MPa com 20 % de β-TCP a 65 % de porosidade; diferença registada a 11 out 2026: o máximo de 6,38 MPa (Wong WS et al. Cureus 2025;17:e86272) foi retirado porque não é rastreável até uma fonte primária do compósito (das cinco referências citadas, quatro são de PCL puro e a quinta, Lim 2011, não dá valores no resumo) e não diz que grandeza é; intervalo anterior 2,2-6,38, típico anterior 4,3 MPa (ponto médio); de fora: 27,9 MPa em Wang 2024, que não é tensão de cedência (o Wang 2024 foi retirado de toda a base a 3 out 2026: Editor Note da revista, ver o módulo); valor anterior: 3-12 MPa (Rezwan K et al. Biomaterials 2006;27); Muito dependente da geometria/porosidade: registar a porosidade do estudo de onde vem o valor; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N175" t="n">
-        <v>4.3</v>
+        <v>2.2</v>
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -14005,27 +14224,32 @@
         </is>
       </c>
       <c r="I178" t="n">
-        <v>12</v>
+        <v>26</v>
       </c>
       <c r="J178" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>Rezwan K et al. Biomaterials 2006;27:3413-3431 (scaffolds ósseos)</t>
+          <t>Zhong M et al. Regen Biomater 2026;13:rbag176 (Discussão e Figura 7E-F)</t>
+        </is>
+      </c>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>https://doi.org/10.1093/rb/rbag176</t>
         </is>
       </c>
       <c r="M178" t="inlineStr">
         <is>
-          <t>a verificar: as fontes divergem e nenhuma mede a reabsorção completa (Yeo 2008, rato, 24 semanas, Mw -89 %; Lam 2009, coelho, 6 meses, perda de massa de cerca de 7 %; só resumo nos dois); Estatuto [confirmar]: fonte clínica a indicar</t>
+          <t>PCL 80 % / β-TCP 20 % por microextrusão (texto completo, PMC13633662): "the degradation of PCL/β-TCP composite scaffold products showed a clear three-stage rule, with a total cycle of about 26 months"; 96,93 % aos 25 meses; ressalvas: estimativa por correlação in vitro / in vivo (envelhecimento acelerado a 50 °C e tíbia de coelho), válida para filamentos de cerca de 220 µm, uma só fonte e um só fabricante; diferença registada a 11 out 2026: intervalo anterior 12-24, típico 18 meses (Rezwan K et al. Biomaterials 2006;27:3413-3431, revisão); outras fontes só com resumo e sem reabsorção completa: Yeo 2008 (rato, 24 semanas, Mw -89 %), Lam 2009 (coelho, 6 meses, perda de massa de cerca de 7 %), Rai 2007 (cão, 33 % dos 6 aos 9 meses); a sensibilidade de 24 a 48 meses (intervalo do PCL) continua no relatório; Estatuto [confirmar]: fonte clínica a indicar</t>
         </is>
       </c>
       <c r="N178" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>A verificar</t>
+          <t>Verificado</t>
         </is>
       </c>
     </row>
@@ -22268,7 +22492,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Limite de fadiga (10^7 ciclos)</t>
+          <t>Resistência à fadiga a 10⁷ ciclos (σmax, R = 0,1)</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -22887,7 +23111,7 @@
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>Problema crítico do docente (2 out 2026): fluoretos em meio ácido, tribocorrosão na ligação implante-pilar, envelhecimento da Y-TZP</t>
+          <t>Problema crítico indicado: fluoretos em meio ácido, tribocorrosão na ligação implante-pilar, envelhecimento da Y-TZP</t>
         </is>
       </c>
     </row>

</xml_diff>